<commit_message>
Fix v2 tables: write real column names so Excel does not remove them
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013PrK8Riv7iDsBQTRwmFryS
</commit_message>
<xml_diff>
--- a/kitting-dashboard/R5B-AMP-Kitting-Control-v2.xlsx
+++ b/kitting-dashboard/R5B-AMP-Kitting-Control-v2.xlsx
@@ -955,19 +955,19 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tblContracts" displayName="tblContracts" ref="A7:M19" headerRowCount="1">
   <autoFilter ref="A7:M19"/>
   <tableColumns count="13">
-    <tableColumn id="1" name="Column1"/>
-    <tableColumn id="2" name="Column2"/>
-    <tableColumn id="3" name="Column3"/>
-    <tableColumn id="4" name="Column4"/>
-    <tableColumn id="5" name="Column5"/>
-    <tableColumn id="6" name="Column6"/>
-    <tableColumn id="7" name="Column7"/>
-    <tableColumn id="8" name="Column8"/>
-    <tableColumn id="9" name="Column9"/>
-    <tableColumn id="10" name="Column10"/>
-    <tableColumn id="11" name="Column11"/>
-    <tableColumn id="12" name="Column12"/>
-    <tableColumn id="13" name="Column13">
+    <tableColumn id="1" name="Contract ID"/>
+    <tableColumn id="2" name="Friendly name"/>
+    <tableColumn id="3" name="Project"/>
+    <tableColumn id="4" name="Top-level assembly code"/>
+    <tableColumn id="5" name="Amps per repeater"/>
+    <tableColumn id="6" name="Total repeaters required"/>
+    <tableColumn id="7" name="Kit-release lead (weeks before final build)"/>
+    <tableColumn id="8" name="AMPS-build lead (weeks before final build)"/>
+    <tableColumn id="9" name="Plan revision"/>
+    <tableColumn id="10" name="Plan updated on"/>
+    <tableColumn id="11" name="Plan updated by"/>
+    <tableColumn id="12" name="Notes"/>
+    <tableColumn id="13" name="Setup check">
       <calculatedColumnFormula>IF(tblContracts[[#This Row],[Contract ID]]="","Missing contract ID",IF(COUNTIF(tblContracts[Contract ID],tblContracts[[#This Row],[Contract ID]])&gt;1,"DUPLICATE contract ID",IF(OR(NOT(ISNUMBER(tblContracts[[#This Row],[Total repeaters required]])),tblContracts[[#This Row],[Total repeaters required]]&lt;=0),"Total repeaters missing",IF(OR(NOT(ISNUMBER(tblContracts[[#This Row],[Kit-release lead (weeks before final build)]])),NOT(ISNUMBER(tblContracts[[#This Row],[AMPS-build lead (weeks before final build)]]))),"Lead time missing",IF(COUNTIF(tblAssemblies[Contract],tblContracts[[#This Row],[Contract ID]])=0,"Assembly setup required","OK")))))</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -979,20 +979,20 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="tblAssemblies" displayName="tblAssemblies" ref="A7:L37" headerRowCount="1">
   <autoFilter ref="A7:L37"/>
   <tableColumns count="12">
-    <tableColumn id="1" name="Column1"/>
-    <tableColumn id="2" name="Column2"/>
-    <tableColumn id="3" name="Column3"/>
-    <tableColumn id="4" name="Column4"/>
-    <tableColumn id="5" name="Column5"/>
-    <tableColumn id="6" name="Column6"/>
-    <tableColumn id="7" name="Column7"/>
-    <tableColumn id="8" name="Column8"/>
-    <tableColumn id="9" name="Column9"/>
-    <tableColumn id="10" name="Column10"/>
-    <tableColumn id="11" name="Column11">
+    <tableColumn id="1" name="Contract"/>
+    <tableColumn id="2" name="Assembly group"/>
+    <tableColumn id="3" name="Assembly code"/>
+    <tableColumn id="4" name="Description"/>
+    <tableColumn id="5" name="Qty per repeater"/>
+    <tableColumn id="6" name="Cumulative supplied to date"/>
+    <tableColumn id="7" name="Updated on"/>
+    <tableColumn id="8" name="Updated by"/>
+    <tableColumn id="9" name="Source reference"/>
+    <tableColumn id="10" name="Correction note"/>
+    <tableColumn id="11" name="Complete sets (calc)">
       <calculatedColumnFormula>IF(AND(ISNUMBER(tblAssemblies[[#This Row],[Qty per repeater]]),tblAssemblies[[#This Row],[Qty per repeater]]&gt;0,tblAssemblies[[#This Row],[Qty per repeater]]=INT(tblAssemblies[[#This Row],[Qty per repeater]])),INT(IF(ISNUMBER(tblAssemblies[[#This Row],[Cumulative supplied to date]]),tblAssemblies[[#This Row],[Cumulative supplied to date]],0)/tblAssemblies[[#This Row],[Qty per repeater]]),"")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" name="Column12">
+    <tableColumn id="12" name="Check (calc)">
       <calculatedColumnFormula>IF(tblAssemblies[[#This Row],[Contract]]="","Missing contract",IF(COUNTIF(tblContracts[Contract ID],tblAssemblies[[#This Row],[Contract]])=0,"Unknown contract",IF(tblAssemblies[[#This Row],[Assembly code]]="","Missing assembly code",IF(COUNTIFS(tblAssemblies[Contract],tblAssemblies[[#This Row],[Contract]],tblAssemblies[Assembly code],tblAssemblies[[#This Row],[Assembly code]])&gt;1,"DUPLICATE contract + code",IF(NOT(AND(ISNUMBER(tblAssemblies[[#This Row],[Qty per repeater]]),tblAssemblies[[#This Row],[Qty per repeater]]&gt;0,tblAssemblies[[#This Row],[Qty per repeater]]=INT(tblAssemblies[[#This Row],[Qty per repeater]]))),"Qty per repeater missing or invalid",IF(tblAssemblies[[#This Row],[Cumulative supplied to date]]="","Supplied total missing",IF(OR(NOT(ISNUMBER(tblAssemblies[[#This Row],[Cumulative supplied to date]])),tblAssemblies[[#This Row],[Cumulative supplied to date]]&lt;0),"Supplied total invalid",IF(tblAssemblies[[#This Row],[Updated on]]="","Not yet updated","OK"))))))))</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1004,14 +1004,14 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="tblPlan" displayName="tblPlan" ref="A6:F152" headerRowCount="1">
   <autoFilter ref="A6:F152"/>
   <tableColumns count="6">
-    <tableColumn id="1" name="Column1"/>
-    <tableColumn id="2" name="Column2"/>
-    <tableColumn id="3" name="Column3"/>
-    <tableColumn id="4" name="Column4"/>
-    <tableColumn id="5" name="Column5">
+    <tableColumn id="1" name="Contract"/>
+    <tableColumn id="2" name="Final build week (Monday)"/>
+    <tableColumn id="3" name="Repeaters planned"/>
+    <tableColumn id="4" name="Note"/>
+    <tableColumn id="5" name="ISO week (calc)">
       <calculatedColumnFormula>IF(ISNUMBER(tblPlan[[#This Row],[Final build week (Monday)]]),"W"&amp;TEXT(_xlfn.ISOWEEKNUM(tblPlan[[#This Row],[Final build week (Monday)]]),"00")&amp;"-"&amp;YEAR(tblPlan[[#This Row],[Final build week (Monday)]]-WEEKDAY(tblPlan[[#This Row],[Final build week (Monday)]],2)+4),"")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" name="Column6">
+    <tableColumn id="6" name="Check (calc)">
       <calculatedColumnFormula>IF(tblPlan[[#This Row],[Contract]]="","Missing contract",IF(COUNTIF(tblContracts[Contract ID],tblPlan[[#This Row],[Contract]])=0,"Unknown contract",IF(NOT(ISNUMBER(tblPlan[[#This Row],[Final build week (Monday)]])),"Missing date",IF(WEEKDAY(tblPlan[[#This Row],[Final build week (Monday)]],2)&lt;&gt;1,"Not a Monday",IF(OR(NOT(ISNUMBER(tblPlan[[#This Row],[Repeaters planned]])),tblPlan[[#This Row],[Repeaters planned]]&lt;0),"Qty missing or invalid","OK")))))</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -7610,7 +7610,7 @@
   </conditionalFormatting>
   <dataValidations count="2">
     <dataValidation sqref="C3" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Check entry" error="Pick a contract from the list (Contracts sheet)." type="list" errorStyle="stop">
-      <formula1>=ContractList</formula1>
+      <formula1>ContractList</formula1>
     </dataValidation>
     <dataValidation sqref="K18" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Check entry" error="Target must be a whole number of repeater kits." type="whole" errorStyle="stop" operator="greaterThanOrEqual">
       <formula1>0</formula1>
@@ -9767,7 +9767,7 @@
   </conditionalFormatting>
   <dataValidations count="3">
     <dataValidation sqref="C3" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Check entry" error="Pick a contract from the list." type="list" errorStyle="stop">
-      <formula1>=ContractList</formula1>
+      <formula1>ContractList</formula1>
     </dataValidation>
     <dataValidation sqref="C5" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Check entry" error="Whole number of weeks (0–520)." type="whole" errorStyle="stop" operator="between">
       <formula1>0</formula1>
@@ -12245,7 +12245,7 @@
   </conditionalFormatting>
   <dataValidations count="4">
     <dataValidation sqref="A8:A5007" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Check entry" error="Pick a contract that exists on the Contracts sheet." type="list" errorStyle="stop">
-      <formula1>=ContractList</formula1>
+      <formula1>ContractList</formula1>
     </dataValidation>
     <dataValidation sqref="E8:E5007" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Check entry" error="Qty per repeater must be a whole number above 0." type="whole" errorStyle="stop" operator="greaterThan">
       <formula1>0</formula1>
@@ -16180,7 +16180,7 @@
   </conditionalFormatting>
   <dataValidations count="3">
     <dataValidation sqref="A7:A5006" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Check entry" error="Pick a contract that exists on the Contracts sheet." type="list" errorStyle="stop">
-      <formula1>=ContractList</formula1>
+      <formula1>ContractList</formula1>
     </dataValidation>
     <dataValidation sqref="B7:B5006" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Monday date required" error="Enter the MONDAY date of the final build week." type="custom" errorStyle="stop">
       <formula1>AND(ISNUMBER(B7),WEEKDAY(B7,2)=1)</formula1>

</xml_diff>